<commit_message>
changed pc_id value in theory question bulk upload and created new api to check all pcIds exists
</commit_message>
<xml_diff>
--- a/public/uploads/sample/bulk_theory_question_sample_file.xlsx
+++ b/public/uploads/sample/bulk_theory_question_sample_file.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" mc:Ignorable="x15 xr xr6 xr10">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20416"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\pc\Desktop\Excel Files\sample files\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\wamp64\www\projects\uatassmt\public\uploads\sample\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{57387578-747E-4473-979A-96212378E394}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D27638AE-3AAD-48DE-A3BD-27323E13A834}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="32760" yWindow="32760" windowWidth="20385" windowHeight="7950"/>
+    <workbookView xWindow="32760" yWindow="32760" windowWidth="20385" windowHeight="7950" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="45" uniqueCount="32">
   <si>
     <t>Question</t>
   </si>
@@ -90,22 +90,40 @@
     <t>8</t>
   </si>
   <si>
-    <t>AMH/N1949_1_PC1</t>
-  </si>
-  <si>
-    <t>AMH/N1949_1_PC1, AMH/N1949_1_PC2</t>
-  </si>
-  <si>
     <t>Updated Wax pattern should be attached to the sprue at an angle of ----------------- to assist in controlling the direction of solidification when casting.</t>
   </si>
   <si>
     <t>5</t>
+  </si>
+  <si>
+    <t>NOS_ID</t>
+  </si>
+  <si>
+    <t>AMH/N1949_1</t>
+  </si>
+  <si>
+    <t>PC1, PC2</t>
+  </si>
+  <si>
+    <t>PC1</t>
+  </si>
+  <si>
+    <t>PC5</t>
+  </si>
+  <si>
+    <t>AMH/N1950_1</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>M</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -444,8 +462,8 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:K3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <dimension ref="A1:L4"/>
   <sheetFormatPr defaultColWidth="12.28515625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="34.140625" style="1" bestFit="1" customWidth="1"/>
@@ -454,11 +472,12 @@
     <col min="8" max="8" width="20.85546875" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="22.42578125" style="1" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="6.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="36.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="12.28515625" style="1"/>
+    <col min="11" max="11" width="13.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="36.5703125" style="1" bestFit="1" customWidth="1"/>
+    <col min="13" max="16384" width="12.28515625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:12" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -490,12 +509,15 @@
         <v>6</v>
       </c>
       <c r="K1" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="L1" s="2" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="2" spans="1:11" ht="75" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:12" ht="75" x14ac:dyDescent="0.25">
       <c r="A2" s="3" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>8</v>
@@ -522,10 +544,13 @@
         <v>19</v>
       </c>
       <c r="K2" s="1" t="s">
-        <v>23</v>
+        <v>25</v>
+      </c>
+      <c r="L2" s="1" t="s">
+        <v>26</v>
       </c>
     </row>
-    <row r="3" spans="1:11" ht="60" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:12" ht="60" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>7</v>
       </c>
@@ -542,7 +567,7 @@
         <v>11</v>
       </c>
       <c r="G3" s="1" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="H3" s="3" t="s">
         <v>12</v>
@@ -554,7 +579,45 @@
         <v>21</v>
       </c>
       <c r="K3" s="1" t="s">
-        <v>22</v>
+        <v>25</v>
+      </c>
+      <c r="L3" s="1" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:12" ht="60" x14ac:dyDescent="0.25">
+      <c r="A4" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="D4" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="E4" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H4" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="I4" s="1" t="s">
+        <v>31</v>
+      </c>
+      <c r="J4" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="K4" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="L4" s="1" t="s">
+        <v>28</v>
       </c>
     </row>
   </sheetData>
@@ -564,7 +627,7 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
@@ -573,7 +636,7 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1"/>
   <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>

</xml_diff>